<commit_message>
Blacklist: 2 entries, 1 depleted
</commit_message>
<xml_diff>
--- a/blacklist.xlsx
+++ b/blacklist.xlsx
@@ -61,6 +61,28 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Satíva</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Draenor (EU)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://raider.io/characters/eu/draenor/Satíva</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>

</xml_diff>